<commit_message>
Close the 2D rounds: results of rounds 6-10, rejection of the impact-ionization factor, eliU report
- STATUS / EXPERIMENTS / ANALYSIS: steps 2-5 finished; larger impact-ionization coefficients diagnosed and
  rejected (with a factor of 5 or more a grounded-body cell cannot hold 1.1 V, against Fig.7(c) of the paper;
  thick bodies latch in the FBE); what the paper's text and Fig.7 / Fig.8 say about the models and about R
- data: tables and raw files of 221 complete runs, the resistor scan, the Id-Vg runs and 12 stopped runs kept
  as evidence; no run of mine is left on the server
- reports: evening section of the 2D report, comparison workbook, status report in eliU form with six
  pictures drawn from my data
- note for Codex in STATUS.md: the disk quota of the shared account ran full 18:14-18:27 and damaged
  CDR_id_i0_idle (from 8.35 ns) and FS_c2_q1300 (no plot files); both need a rerun

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/claude/reports/GT_IRPS2026_논문대비_비교표_2026-10-06.xlsx
+++ b/claude/reports/GT_IRPS2026_논문대비_비교표_2026-10-06.xlsx
@@ -831,12 +831,12 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>t_A에 몸체 정공 약 1300개(0.21 fC)를 조건으로 넣으면 200 ns 손실 82 / 56 / 16.6 / 12.5 / 1.6 mV (논문 100 / 50 / 14.6 / 7 / 1), 꺾이는 모양도 같음. 정공의 출처는 재현 안 됨</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>근접</t>
+          <t>최종 구성: t_A에 몸체 정공 약 1050개(0.17 fC, Fig. 8(a) 막대)를 조건으로 넣으면 첫 구간 2.6 / 2.2 / 1.1 / 1.1 / 0.13 mV (논문 55 / 29 / 7.1 / 3.5 / 0), 200 ns 20 / 15.5 / 6.2 / 5.4 / 1.6 mV (논문 100 / 50 / 14.6 / 7 / 1). Case 순서와 Case 5는 맞음. 전하 1.25배(약 1300개)에서는 82 / 56 / 16.6 / 12.5 / 1.6 mV. 정공의 출처는 재현 안 됨</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>불일치</t>
         </is>
       </c>
     </row>
@@ -853,12 +853,12 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>막대 = 공통 최종 전위 − 공핍 몸체 전위임을 확인. 정공 약 1050개면 548 / 442 / 363 / 319 / 367 mV (논문 555 / 445 / 365 / 320 / 368). 손실에 맞춘 전하에서는 53~68 mV 높음</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>근접</t>
+          <t>막대 = 공통 최종 전위 − 공핍 몸체 전위로 읽힘. 최종 구성(정공 약 1050개)에서 548 / 442 / 363 / 319 / 367 mV (논문 555 / 445 / 365 / 320 / 368). 정공 전하는 조건으로 넣은 값(대리 생성 + 저장 노드 1.1 V 유지)</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>일치</t>
         </is>
       </c>
     </row>
@@ -875,7 +875,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Z–Z'만 R 2e5 Ω에서 크기가 나옴(0.0093 대 0.0100, 쌓이지 않는 이동). Y–Y' 0.0007~0.0015 대 0.0535, 충돌 이온화 켠 Z–Z'의 급락은 안 나옴</t>
+          <t>최종 구성(이상적 WL): Y–Y' 0.0014 대 0.0535, Z–Z' 0.0014 대 0.0100 mV/사이클, 충돌 이온화 켠 Z–Z'의 급락은 안 나옴(몸체를 665 mV 수준으로 충전해도). WL 저항 200 kΩ은 첫 사이클에 한 번 이동할 뿐 쌓이지 않고 쓰기를 깨뜨려 쓰지 않음</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>2D 소자 확정: Id–Vg·쓰기·FBE 손실은 판독 오차 안(FBE는 몸체 정공 전하를 조건으로 넣은 결과). 남은 것: 정공의 출처, 로우 해머 Y–Y'와 Fig. 7(a)</t>
+          <t>2D 구성 fin2(사용자 결정 반영): Id–Vg·쓰기·몸체 전위(조건)는 판독 오차 안. FBE 손실은 Case 순서가 맞고 첫 구간 크기가 3~20배 작음. 남은 것: 정공의 출처, 막대와 손실의 동시 일치, 로우 해머 Y–Y'와 Fig. 7(a)</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -942,7 +942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G127"/>
+  <dimension ref="A1:G136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="G116" s="3" t="inlineStr">
         <is>
-          <t>과도 해석의 저장 노드 용량을 1.8 fF로 확정(점수 6.49 → 0.93). 두 번째 근거: BL 1.168 V로 쓰면 WL이 꺼진 뒤 1.08 V, 논문 곡선 시작값 1.1 V. 본문 값은 감지 여유 계산용으로 유지</t>
+          <t>과도 해석의 저장 노드 용량을 1.8 fF로 확정(점수 6.49 → 0.93). 근거는 쓰기 곡선의 전하 수지: 4.2 fF × 0.72 V ÷ 12 ps = 252 µA가 필요한데 Fig. 5(c) 최대 전류가 229 µA. (WL이 꺼진 뒤 노드가 내려앉는 값은 독립 근거가 아니어서 뺌.) 본문 값은 감지 여유 계산용으로 유지</t>
         </is>
       </c>
     </row>
@@ -5251,12 +5251,12 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>2D 완성: FBE, 몸체를 막대 전위로 (조건)</t>
+          <t>2D 완성: FBE, 몸체를 막대 전위로 (조건, 최종 구성 fin2)</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>첫 저전위 구간 / 200 ns 손실: Case 1~5 (1.8 fF)</t>
+          <t>첫 저전위 구간 / 200 ns 손실: Case 1~5 (1.8 fF, A 1.7e21)</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
@@ -5266,7 +5266,7 @@
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>2.6 / 2.0 / 0.98 / 1.02 / 0.13 mV, 19.8 / 14.4 / 5.8 / 5.1 / 1.6 mV</t>
+          <t>2.62 / 2.16 / 1.06 / 1.09 / 0.13 mV, 20.3 / 15.5 / 6.2 / 5.4 / 1.6 mV</t>
         </is>
       </c>
       <c r="E120" s="3" t="inlineStr">
@@ -5281,14 +5281,14 @@
       </c>
       <c r="G120" s="3" t="inlineStr">
         <is>
-          <t>Case 순서와 Case 5는 맞음. 뒤쪽 구간의 구간당 손실은 논문과 2배 이내. 곡선이 꺾이지 않음. 정공은 몸체 영역의 일정 생성으로 넣고 그동안 저장 노드를 1.1 V로 붙잡음(대리 수단)</t>
+          <t>사용자 결정(2026-10-06): 정공 전하는 조건으로 두고 Fig. 8(a) 막대에 맞춤. 몸체 상승 548 / 442 / 363 / 319 / 367 mV(점수 0.12). 실행 Dh1F_c1~c5. Case 순서와 Case 5는 맞음. 뒤쪽 구간의 구간당 손실은 논문과 2배 이내. 곡선이 꺾이지 않음. 정공은 몸체 영역의 일정 생성으로 넣고 그동안 저장 노드를 1.1 V로 붙잡음(대리 수단)</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>2D 완성: FBE, 정공 전하 1.25배 (최종)</t>
+          <t>2D 완성: FBE, 정공 전하 1.25배 (참고)</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
@@ -5325,7 +5325,7 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>2D 완성: FBE, 정공 전하 1.25배 (최종)</t>
+          <t>2D 완성: FBE, 정공 전하 1.25배 (참고)</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
@@ -5362,7 +5362,7 @@
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>2D 완성: FBE, 정공 전하 1.25배 (최종)</t>
+          <t>2D 완성: FBE, 정공 전하 1.25배 (참고)</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
@@ -5399,7 +5399,7 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>2D 완성: FBE, 정공 전하 1.25배 (최종)</t>
+          <t>2D 완성: FBE, 정공 전하 1.25배 (참고)</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
@@ -5541,6 +5541,339 @@
       <c r="G127" s="3" t="inlineStr">
         <is>
           <t>저장 노드 1.8 fF 기준. R 2e5 Ω을 넣으면 Z–Z' 0.0093, 접지 0.0196 mV(10사이클 평균)</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
+          <t>2D 완성: WL 저항 200 kΩ의 문제점</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>쓰기 곡선 12 / 24 / 39 / 60 ps (R을 WL 경로에 둘 때, Case 2)</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>0.72 / 0.92 / 1.06 / 1.13 V</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>0.07 / 0.22 / 0.51 / 0.88 V</t>
+        </is>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>점수 0.93 → 18.85</t>
+        </is>
+      </c>
+      <c r="F128" s="6" t="inlineStr">
+        <is>
+          <t>불일치</t>
+        </is>
+      </c>
+      <c r="G128" s="3" t="inlineStr">
+        <is>
+          <t>게이트 노드가 1.7 V에 닿는 데 60 ps. 사용자 결정(문제가 없을 때만 사용)에 따라 쓰지 않음. 논문 Fig. 7(b)에는 R이 victim 게이트 노드와 WL 전원 사이에 그려져 있고 값은 없음. 실행 DraW_c2</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>2D 완성: WL 저항 200 kΩ의 문제점</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>Z–Z' 손실이 쌓이는지: 1사이클 뒤 / 10사이클 뒤 (4.2 fF, 충돌 이온화 끔)</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>0.0100 mV/사이클</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>−0.0929 / −0.0930 mV. 1.8 fF: 첫 사이클 −0.203 mV. 몸체 접지: −0.190 / −0.196 mV (1.8 fF −0.445 / −0.454)</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>첫 사이클 한 번, 누적 없음</t>
+        </is>
+      </c>
+      <c r="F129" s="6" t="inlineStr">
+        <is>
+          <t>불일치</t>
+        </is>
+      </c>
+      <c r="G129" s="3" t="inlineStr">
+        <is>
+          <t>움직이는 전하가 용량과 무관하게 일정(부유 0.37~0.39 aC, 접지 0.80 aC). Codex의 50사이클·idle 대조: 0.1001 → 0.1050 mV. '10사이클 평균 0.0100'은 4.2 fF에서 이 이동을 10으로 나눈 값. 실행 Dr2R*, DtcR*</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>2D 완성: 몸체가 충전된 로우 해머</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>10사이클 변화, Y–Y' / Z–Z': 정공 1056개(445 mV), 1970개(665 mV). 충돌 이온화 켬, 이상적 WL</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>Z–Z' 급락 (1.1 → 0.58 V)</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>+0.020 / +0.023 mV, +0.038 / +0.029 mV</t>
+        </is>
+      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>급락 없음</t>
+        </is>
+      </c>
+      <c r="F130" s="6" t="inlineStr">
+        <is>
+          <t>불일치</t>
+        </is>
+      </c>
+      <c r="G130" s="3" t="inlineStr">
+        <is>
+          <t>몸체를 Fig. 8(a), Fig. 7(e) 수준으로 충전해도 노드가 내려가지 않음. 실행 DhaR*, DhcR*</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>2D 완성: Y–Y' 후보</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>마지막 5사이클 손실: 기준 / BL 직렬 저항 10 kΩ / + aggressor 노드 1.1 V / WL 저항 200 kΩ</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>0.0535 mV/사이클</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>0.00144 / 0.00144 / 0.00144 / 0.00137 mV</t>
+        </is>
+      </c>
+      <c r="E131" s="3" t="inlineStr">
+        <is>
+          <t>약 37배 작음</t>
+        </is>
+      </c>
+      <c r="F131" s="6" t="inlineStr">
+        <is>
+          <t>불일치</t>
+        </is>
+      </c>
+      <c r="G131" s="3" t="inlineStr">
+        <is>
+          <t>어느 후보도 값을 움직이지 않음. 남는 값은 정적 누설(용량에 반비례). 실행 DfinRy_yy, DybRy_yy, DydRy_yy, DtcRy_yy</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="3" t="inlineStr">
+        <is>
+          <t>2D 완성: 가정 민감도 (Case 2)</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>스페이서 SiO2 / HfO2 / BL 기둥 50 nm: 쓰기 12 ps, GIDL log10 I, FBE 첫 구간 손실</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>0.72 V, −13.2, 29 mV</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>0.72 / 0.79 / 0.74 V, −13.37 / −12.81 / −13.27, 2.32 / 1.84 / 2.15 mV (기준 0.74 V, −13.24, 2.16 mV)</t>
+        </is>
+      </c>
+      <c r="E132" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F132" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G132" s="3" t="inlineStr">
+        <is>
+          <t>좋아지는 점수 없음. Si3N4 스페이서와 100 nm 기둥 유지. 이동도에 수직 전계 의존을 넣으면 문턱은 같고 과도 해석이 WL 상승 에지에서 수렴하지 않음. 실행 Dsx*, Dsh*, Dbw*, Dm1I_c2</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>2D 완성: 충돌 이온화 계수 배수 (진단)</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>WL 꺼진 뒤 몸체에 남는 정공, 배수 1 / 5 / 7 / 10 (Case 2)</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>막대에 해당하는 값 1056개</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>35 / 119 / 1334 / 2349개</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="inlineStr">
+        <is>
+          <t>5배와 7배 사이에 문턱</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G133" s="3" t="inlineStr">
+        <is>
+          <t>배수는 출처가 없는 진단값(채택 안 함). 7배: Case 1~5 1462 / 1334 / 1302 / 1320 / 1969개, 유지 구간 처짐 없음, WL 꺼짐에서 노드 −151 ~ −207 mV. 실행 Dj*F, Di1F</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="3" t="inlineStr">
+        <is>
+          <t>2D 완성: 충돌 이온화 계수 배수 (진단)</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>대리 생성 없이 FBE, 7배: 첫 구간 / 200 ns 손실, Case 3 / Case 5</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>7.1 / 14.6 mV, 0 / 1 mV</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>9.5 / 29.9 mV, 0.17 / 1.60 mV</t>
+        </is>
+      </c>
+      <c r="E134" s="3" t="inlineStr">
+        <is>
+          <t>Case 3 +34 % / 2.0배</t>
+        </is>
+      </c>
+      <c r="F134" s="7" t="inlineStr">
+        <is>
+          <t>근접</t>
+        </is>
+      </c>
+      <c r="G134" s="3" t="inlineStr">
+        <is>
+          <t>Case 1, 2는 BL이 0 V가 되면 1 ns 안에 0.58~0.63 V가 빠짐(래치). 6배: Case 4는 애벌랜치 없음(18개), Case 2 753개·0.38 mV, Case 5 1086개·355 mV·0.12 mV. Case마다 문턱이 달라 Fig. 8 전체를 설명하지 못함. 실행 Dk6F, Dk7F</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="3" t="inlineStr">
+        <is>
+          <t>2D 완성: 충돌 이온화 계수 배수 (기각 근거)</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>몸체를 접지한 셀의 저장 노드: 쓰기 중 / 해머 시작 전, 기본 / 5배 / 7배</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>접지 몸체 + 충돌 이온화 켬에서 1.1 V 유지 (Fig. 7(c), 0.036 mV/사이클)</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>0.83 / 1.055 V, 0.08 / 0.096 V, −0.19 / −0.27 V</t>
+        </is>
+      </c>
+      <c r="E135" s="3" t="inlineStr">
+        <is>
+          <t>5배 이상에서 '1'을 유지하지 못함</t>
+        </is>
+      </c>
+      <c r="F135" s="6" t="inlineStr">
+        <is>
+          <t>불일치</t>
+        </is>
+      </c>
+      <c r="G135" s="3" t="inlineStr">
+        <is>
+          <t>몸체가 0 V에 묶이면 애벌랜치를 멈출 것이 없어 N+/p 접합이 1.1 V에서 항복. 논문의 충돌 이온화는 이만큼 강하지 않음 → 계수 배수 기각. 실행 DtcRzg_zz, Dw5Rzg_zz, Dw7Rzg_zz, Du7Rzg_zz, Du9Rzg_zz</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>2D 완성: 충돌 이온화 계수 배수 (진단)</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>최종 구성(막대 전하 조건)에 4배 / 5배: 첫 구간 손실 Case 3 / Case 4</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>7.1 / 3.5 mV</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>26.5 / 17.1 mV, 78.9 / 37.1 mV</t>
+        </is>
+      </c>
+      <c r="E136" s="3" t="inlineStr">
+        <is>
+          <t>정공도 1.5~2배로 늘어남</t>
+        </is>
+      </c>
+      <c r="F136" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G136" s="3" t="inlineStr">
+        <is>
+          <t>대리 생성 자체가 증폭돼 막대 전하가 유지되지 않음(4배에서 1630 / 1736 / 1630 / 1405 / 1970개). 같은 정공 수에서 기본 계수보다 Case 3 1.6배·3.0배, Case 4 1.5배·2.2배. Case 1, 2는 래치. 실행 Dv4F, Dv5F</t>
         </is>
       </c>
     </row>
@@ -15612,7 +15945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -16664,57 +16997,513 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>15시</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>fin</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>1.8 fF + A 1.7e21 + 정공 전하 1.25배 (16개 실행)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>0.73</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>0.93</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>2.03</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>0.84</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>0.51</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>11.9</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>참고 (손실에 맞춘 전하)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>ra</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>WL 저항 200 kΩ을 쓰기·FBE에</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>18.85</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>0.24</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>3.14</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>1.60</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>기각 (쓰기가 깨짐)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>4, 6</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>r2 / tc</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>WL 저항 200 kΩ 로우 해머 (4.2 fF / 1.8 fF)</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>첫 사이클 −0.093 / −0.203 mV 뒤 평탄</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>급락 없음</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>기각 (누적 없음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>sx / sh / bw</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>스페이서 SiO2 / HfO2, BL 기둥 50 nm (Case 2)</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Case 2 문턱 같음</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>1.17 / 1.35 / 0.94</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>444 / 438 / 442 mV</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>2.32 / 1.84 / 2.15 mV</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>16.3 / 13.7 / 13.8 mV</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>기본 유지</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>ha / hc</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>몸체 충전(1056 / 1970개) 뒤 로우 해머</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>손실 없음</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>급락 없음</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>재현 안 됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>yb / yd</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Y–Y': BL 직렬 저항 10 kΩ, aggressor 노드 1.1 V</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>0.00144 (변화 없음)</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>영향 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>5~7</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>j2~j7, i1, k6, k7</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>충돌 이온화 계수 × 2~10, 대리 생성 없음 (진단)</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>×7: 651 / 516 / 416 / 409 / 566 mV</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>×7: Case 3 9.5 mV, Case 1·2 래치</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>×7: Case 3 29.9 mV</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>진단 (채택 안 함)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>v4 / v5</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>최종 구성 + 계수 × 4 / × 5 (진단)</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>690 ~ 430 / 744 ~ 476 mV</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Case 3 26.5 / 78.9 mV, Case 1·2 래치</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>진단 (대리 생성이 증폭됨)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>fin</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>1.8 fF + A 1.7e21 + 정공 전하 1.25배 (16개 실행)</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>fin2</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>사용자 결정: 1.8 fF + A 1.7e21 + 정공 전하 1.0배(Fig. 8(a) 막대), 이상적 WL</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>0.73</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>0.93</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>2.03</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>0.84</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>0.51</t>
-        </is>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>4.4</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>2.97</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>1.44</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>4.39</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
         <is>
           <t>11.9</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
-        <is>
-          <t>확정</t>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>확정 (사용자 결정)</t>
         </is>
       </c>
     </row>

</xml_diff>